<commit_message>
otimiza snippets de custo-benefício e mesa de vidro
</commit_message>
<xml_diff>
--- a/docs/SEO_MASTER_Casa_Pratica.xlsx
+++ b/docs/SEO_MASTER_Casa_Pratica.xlsx
@@ -225,8 +225,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterSEO" displayName="MasterSEO" ref="A1:S13" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:S13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MasterSEO" displayName="MasterSEO" ref="A1:S14" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:S14"/>
   <tableColumns count="19">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Grupo / Silo"/>
@@ -276,8 +276,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="HistoricoAcoes" displayName="HistoricoAcoes" ref="A1:J3" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:J2"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="HistoricoAcoes" displayName="HistoricoAcoes" ref="A1:J7" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:J7"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Data"/>
     <tableColumn id="2" name="ID"/>
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S13"/>
+  <dimension ref="A1:S14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -831,7 +831,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>Acompanhar</t>
+          <t>Otimizar</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
@@ -841,24 +841,36 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Em monitoramento</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="n"/>
-      <c r="N3" s="3" t="n"/>
+          <t>Alterado / monitorando</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="n">
+        <v>46268</v>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>SEO on-page — Etapa 1</t>
+        </is>
+      </c>
       <c r="O3" s="4">
         <f>IF([@[Última alteração]]="","",[@[Última alteração]]+28)</f>
         <v/>
       </c>
-      <c r="P3" s="3" t="n"/>
-      <c r="Q3" s="3" t="n"/>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Alteração realizada</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>62</v>
+      </c>
       <c r="R3" s="3">
         <f>IF(OR([@[Posição atual]]="",[@[Posição anterior]]=""),"",[@[Posição anterior]]-[@[Posição atual]])</f>
         <v/>
       </c>
       <c r="S3" s="3" t="inlineStr">
         <is>
-          <t>Intenção comercial específica.</t>
+          <t>Etapa 1 — consolidação da intenção custo-benefício/preço-performance. Home permanece dona do ranking geral de melhores fogões 5 bocas. Intervenção limitada a title e meta description. Aguardar recrawl/GSC antes de nova intervenção.</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1269,7 @@
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>Mapear</t>
+          <t>Otimizar</t>
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr">
@@ -1267,16 +1279,26 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Mapeado</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="n"/>
-      <c r="N9" s="3" t="n"/>
+          <t>Alterado / monitorando</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="n">
+        <v>46268</v>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>SEO on-page — Etapa 1</t>
+        </is>
+      </c>
       <c r="O9" s="4">
         <f>IF([@[Última alteração]]="","",[@[Última alteração]]+28)</f>
         <v/>
       </c>
-      <c r="P9" s="3" t="n"/>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>Alteração realizada</t>
+        </is>
+      </c>
       <c r="Q9" s="3" t="n"/>
       <c r="R9" s="3">
         <f>IF(OR([@[Posição atual]]="",[@[Posição anterior]]=""),"",[@[Posição anterior]]-[@[Posição atual]])</f>
@@ -1284,7 +1306,7 @@
       </c>
       <c r="S9" s="3" t="inlineStr">
         <is>
-          <t>Decisão comparativa entre materiais.</t>
+          <t>Etapa 1 — alterados somente title e meta description para consolidar a intenção "fogão com mesa de vidro ou inox". Blog /blog/fogao-mesa-de-vidro-ou-inox/ permanece URL dona da comparação vidro × inox; hub /melhores/melhor-fogao-mesa-de-vidro/ permanece dono de “melhor fogão mesa de vidro”. Aguardar recrawl/GSC antes de nova intervenção.</t>
         </is>
       </c>
     </row>
@@ -1549,6 +1571,91 @@
       <c r="S13" s="3" t="inlineStr">
         <is>
           <t>Consulta ampla; precisa de contexto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Segurança / risco — mesa de vidro</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>fogão com mesa de vidro é perigoso</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>fogão com mesa de vidro é seguro?; pode estourar</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Informacional</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>/blog/fogao-mesa-de-vidro-seguro/</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>/blog/fogao-mesa-de-vidro-seguro/</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Otimizar</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Alterado / monitorando</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="n">
+        <v>46268</v>
+      </c>
+      <c r="N14" s="3" t="inlineStr">
+        <is>
+          <t>SEO on-page — Etapa 1</t>
+        </is>
+      </c>
+      <c r="O14" s="4">
+        <f>IF([@[Última alteração]]="","",[@[Última alteração]]+28)</f>
+        <v/>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Alteração realizada</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="R14" s="3">
+        <f>IF(OR([@[Posição atual]]="",[@[Posição anterior]]=""),"",[@[Posição anterior]]-[@[Posição atual]])</f>
+        <v/>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>Etapa 1 executada somente em title e meta description para consolidar a intenção de segurança/risco (“é perigoso”). Página já existente e dona da intenção. Comparativo vidro × inox permanece separado como intenção de comparação; hub mesa de vidro permanece dono do ranking. Aguardar recrawl/GSC antes de nova intervenção.</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1963,6 +2070,132 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>Variação volume: keyword principal 590 (tamanho fogão 5 bocas) + variação 90 (tamanho do fogão 5 bocas). Próxima revisão: ~01/10/2026. Sem commit/push/deploy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>melhor fogao 5 bocas custo beneficio</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>/fogao-5-bocas-custo-beneficio/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SEO on-page — Etapa 1</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>62</v>
+      </c>
+      <c r="G5" t="n">
+        <v>62</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Title e meta description da página otimizados para consolidar a intenção de custo-benefício/preço-performance.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Alteração realizada</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Home permanece dona de “melhores fogões 5 bocas”; esta URL permanece dona da intenção específica de custo-benefício. Aguardar recrawl/GSC antes de nova intervenção.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>fogão com mesa de vidro ou inox</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>/blog/fogao-mesa-de-vidro-ou-inox/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SEO on-page — Etapa 1</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>title e meta description</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Alteração realizada</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>comparação vidro × inox permanece separada do ranking de melhores fogões com mesa de vidro; aguardar recrawl/GSC antes de nova intervenção.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="n">
+        <v>46268</v>
+      </c>
+      <c r="B7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>fogão com mesa de vidro é perigoso</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>/blog/fogao-mesa-de-vidro-seguro/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>SEO on-page — Etapa 1</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>13</v>
+      </c>
+      <c r="G7" t="n">
+        <v>13</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Title + meta description</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Alteração realizada</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Consolidação da intenção de segurança/risco; comparativo vidro × inox e hub de ranking permanecem com suas respectivas intenções.</t>
         </is>
       </c>
     </row>

</xml_diff>